<commit_message>
Atualiza historico e state 2026-05-17 14:24 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Resumo" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$K$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$K$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -47,12 +47,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDE2E2"/>
+        <fgColor rgb="00FFF4CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF4CE"/>
+        <fgColor rgb="00FDE2E2"/>
       </patternFill>
     </fill>
   </fills>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -519,12 +519,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -539,102 +539,98 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Deferimento RJ</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>RJ</t>
-        </is>
-      </c>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>4ce791b96b8e30d6</t>
+          <t>4a32518f78fb004d</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-13T19:28:37</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-05T00:00:00</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>47508411000156</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>00776574000156</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Comunicado ao Mercado</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Notícia veiculada na mídia</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Apresentações a analistas/agentes do mercado</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Apresentação de Resultados 1T26</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>média</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr"/>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>7f505e05b533c1cb</t>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>c7abdd8cf1173c78</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -649,91 +645,682 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
-        </is>
-      </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>alta</t>
+          <t>média</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>430d875fcf9deef3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Assembleia</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>4c0a5e94fef4fcac</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Assembleia</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>4c0a5e94fef4fcac</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Aviso aos Acionistas</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>baixa</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>77d6445a8533898f</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Apresentações a analistas/agentes do mercado</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Apresentação de Resultado - 1T26</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>887face2818a9f45</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>renúncia</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>7e01f0ddc31fe98d</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Convocação AGE</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr"/>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>21436dade51d1f6f</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13T00:00:00</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>00776574000156</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Alienação de Ativos HNT São Paulo</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>b89c74a63ef45b3f</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13T00:00:00</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>GRUPO CASAS BAHIA S.A.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>33041260065290</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Apresentações a analistas/agentes do mercado</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Apresentação de Resultado 1T26</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>382bf745755fc687</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>CVLB BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>16233389000155</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Deferimento RJ</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>4ce791b96b8e30d6</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Notícia veiculada na mídia</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>7f505e05b533c1cb</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr"/>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K15" s="3" t="inlineStr">
         <is>
           <t>caa180472807662d</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>2026-05-13T19:28:37</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>2026-05-04T00:00:00</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>00776574000156</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Comunicado ao Mercado</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>CAM 268 24 - Desistência dos requerentes</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>média</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr"/>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>21a22f76b5882ca9</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K5"/>
+  <autoFilter ref="A1:K16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -744,7 +1331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -788,16 +1375,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
@@ -810,13 +1397,13 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -829,12 +1416,31 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GRUPO CASAS BAHIA S.A.</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-05-24 14:22 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Resumo" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$K$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$K$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -517,92 +517,92 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17T14:24:03</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15T00:00:00</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>CVLB BRASIL S.A.</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>16233389000155</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Assembleia</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>AGE</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Alteração Estatuto Social</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>média</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>4a32518f78fb004d</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-05-24T14:22:09</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-05-22T00:00:00</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>00776574000156</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Aviso aos Acionistas</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Outros avisos</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>baixa</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>08a01e6ba0b6a7b7</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -613,24 +613,24 @@
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>c7abdd8cf1173c78</t>
+          <t>02427520e01022e3</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-20T00:00:00</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -645,17 +645,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Venda da Participação Societária na Stix</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -666,49 +666,49 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>430d875fcf9deef3</t>
+          <t>84630037d40074aa</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-18T00:00:00</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -719,12 +719,12 @@
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>4c0a5e94fef4fcac</t>
+          <t>3942bd4b6cc31f40</t>
         </is>
       </c>
     </row>
@@ -736,17 +736,17 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -761,7 +761,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -772,12 +772,12 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>4c0a5e94fef4fcac</t>
+          <t>4a32518f78fb004d</t>
         </is>
       </c>
     </row>
@@ -1005,7 +1005,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1025,12 +1025,12 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Alienação de Ativos HNT São Paulo</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1041,12 +1041,12 @@
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>b89c74a63ef45b3f</t>
+          <t>c7abdd8cf1173c78</t>
         </is>
       </c>
     </row>
@@ -1058,32 +1058,32 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1094,81 +1094,77 @@
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>382bf745755fc687</t>
+          <t>4c0a5e94fef4fcac</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-13T19:28:37</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-05T00:00:00</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>CVLB BRASIL S.A.</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>16233389000155</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>Fato Relevante</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Deferimento RJ</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>RJ</t>
-        </is>
-      </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
-        </is>
-      </c>
-      <c r="K13" s="3" t="inlineStr">
-        <is>
-          <t>4ce791b96b8e30d6</t>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Assembleia</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>4c0a5e94fef4fcac</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1183,17 +1179,17 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Notícia veiculada na mídia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1204,77 +1200,77 @@
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>7f505e05b533c1cb</t>
+          <t>430d875fcf9deef3</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-13T19:28:37</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-05T00:00:00</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>47508411000156</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>Fato Relevante</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="I15" s="3" t="inlineStr"/>
-      <c r="J15" s="3" t="inlineStr">
-        <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
-        </is>
-      </c>
-      <c r="K15" s="3" t="inlineStr">
-        <is>
-          <t>caa180472807662d</t>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13T00:00:00</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>GRUPO CASAS BAHIA S.A.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>33041260065290</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Apresentações a analistas/agentes do mercado</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Apresentação de Resultado 1T26</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>382bf745755fc687</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1299,7 +1295,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>CAM 268 24 - Desistência dos requerentes</t>
+          <t>Alienação de Ativos HNT São Paulo</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1310,17 +1306,233 @@
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>b89c74a63ef45b3f</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>CVLB BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>16233389000155</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Deferimento RJ</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>4ce791b96b8e30d6</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Notícia veiculada na mídia</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>7f505e05b533c1cb</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr"/>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>caa180472807662d</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-04T00:00:00</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>00776574000156</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>CAM 268 24 - Desistência dos requerentes</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>21a22f76b5882ca9</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K16"/>
+  <autoFilter ref="A1:K20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1331,7 +1543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1378,13 +1590,13 @@
         <v>3</v>
       </c>
       <c r="C2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -1397,13 +1609,13 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -1419,10 +1631,10 @@
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -1441,6 +1653,25 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MARISA LOJAS SA</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-05-25 15:46 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -782,55 +782,55 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>2026-05-17T14:24:03</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>2026-05-14T00:00:00</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>47508411000156</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Aviso aos Acionistas</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Assembleia</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>baixa</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>77d6445a8533898f</t>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>430d875fcf9deef3</t>
         </is>
       </c>
     </row>
@@ -857,17 +857,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -878,228 +878,228 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>887face2818a9f45</t>
+          <t>4c0a5e94fef4fcac</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>2026-05-17T14:24:03</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>2026-05-14T00:00:00</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>47508411000156</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Assembleia</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>4c0a5e94fef4fcac</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>00776574000156</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Comunicado ao Mercado</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Apresentações a analistas/agentes do mercado</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Apresentação de Resultados 1T26</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>c7abdd8cf1173c78</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Convocação AGE</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>21436dade51d1f6f</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>renúncia</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="J12" s="3" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="K12" s="3" t="inlineStr">
         <is>
           <t>7e01f0ddc31fe98d</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-17T14:24:03</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-14T00:00:00</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>47508411000156</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>Fato Relevante</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Convocação AGE</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr"/>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>21436dade51d1f6f</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17T14:24:03</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-14T00:00:00</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>00776574000156</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Comunicado ao Mercado</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Apresentação de Resultados 1T26</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>média</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>c7abdd8cf1173c78</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17T14:24:03</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-14T00:00:00</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>47508411000156</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Assembleia</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>AGE</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>média</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>4c0a5e94fef4fcac</t>
         </is>
       </c>
     </row>
@@ -1126,17 +1126,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1147,65 +1147,65 @@
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>4c0a5e94fef4fcac</t>
+          <t>887face2818a9f45</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>2026-05-17T14:24:03</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>2026-05-14T00:00:00</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>47508411000156</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Assembleia</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>AGE</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Aviso aos Acionistas</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>média</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>430d875fcf9deef3</t>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>baixa</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>77d6445a8533898f</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-05-26 16:38 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -782,55 +782,55 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>2026-05-17T14:24:03</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>2026-05-14T00:00:00</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>47508411000156</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Assembleia</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>AGE</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Aviso aos Acionistas</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>média</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>430d875fcf9deef3</t>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>baixa</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>77d6445a8533898f</t>
         </is>
       </c>
     </row>
@@ -857,17 +857,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -878,228 +878,228 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
+          <t>887face2818a9f45</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>renúncia</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>7e01f0ddc31fe98d</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Convocação AGE</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr"/>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>21436dade51d1f6f</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>00776574000156</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Apresentações a analistas/agentes do mercado</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Apresentação de Resultados 1T26</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>c7abdd8cf1173c78</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Assembleia</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
           <t>4c0a5e94fef4fcac</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17T14:24:03</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-14T00:00:00</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>47508411000156</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Assembleia</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>AGE</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>média</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>4c0a5e94fef4fcac</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17T14:24:03</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-14T00:00:00</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>00776574000156</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Comunicado ao Mercado</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Apresentação de Resultados 1T26</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>média</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>c7abdd8cf1173c78</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-17T14:24:03</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-14T00:00:00</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>47508411000156</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>Fato Relevante</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>Convocação AGE</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="inlineStr"/>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
-        </is>
-      </c>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
-          <t>21436dade51d1f6f</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-17T14:24:03</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-14T00:00:00</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>47508411000156</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>Comunicado ao Mercado</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>renúncia</t>
-        </is>
-      </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
-        <is>
-          <t>7e01f0ddc31fe98d</t>
         </is>
       </c>
     </row>
@@ -1126,17 +1126,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1147,65 +1147,65 @@
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>887face2818a9f45</t>
+          <t>4c0a5e94fef4fcac</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>2026-05-17T14:24:03</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>2026-05-14T00:00:00</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>47508411000156</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Aviso aos Acionistas</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Assembleia</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>baixa</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>77d6445a8533898f</t>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>430d875fcf9deef3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-05-27 16:34 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -782,55 +782,55 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>2026-05-17T14:24:03</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>2026-05-14T00:00:00</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>47508411000156</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Aviso aos Acionistas</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Assembleia</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>baixa</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>77d6445a8533898f</t>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>430d875fcf9deef3</t>
         </is>
       </c>
     </row>
@@ -857,17 +857,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -878,228 +878,228 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>887face2818a9f45</t>
+          <t>4c0a5e94fef4fcac</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>2026-05-17T14:24:03</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>2026-05-14T00:00:00</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>47508411000156</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Assembleia</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>4c0a5e94fef4fcac</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>00776574000156</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Comunicado ao Mercado</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Apresentações a analistas/agentes do mercado</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Apresentação de Resultados 1T26</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>média</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>c7abdd8cf1173c78</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Convocação AGE</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>21436dade51d1f6f</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>alta</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>renúncia</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="J12" s="3" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="K12" s="3" t="inlineStr">
         <is>
           <t>7e01f0ddc31fe98d</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-17T14:24:03</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-14T00:00:00</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>47508411000156</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>Fato Relevante</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Convocação AGE</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>alta</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr"/>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>21436dade51d1f6f</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17T14:24:03</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-14T00:00:00</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>00776574000156</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Comunicado ao Mercado</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Apresentação de Resultados 1T26</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>média</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>c7abdd8cf1173c78</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-17T14:24:03</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-14T00:00:00</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>47508411000156</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Assembleia</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>AGE</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>média</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>4c0a5e94fef4fcac</t>
         </is>
       </c>
     </row>
@@ -1126,17 +1126,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1147,65 +1147,65 @@
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>4c0a5e94fef4fcac</t>
+          <t>887face2818a9f45</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>2026-05-17T14:24:03</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>2026-05-14T00:00:00</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>47508411000156</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Assembleia</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>AGE</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Aviso aos Acionistas</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
         <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>média</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>430d875fcf9deef3</t>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>baixa</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>77d6445a8533898f</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-05-28 16:44 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -715,12 +715,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -757,22 +757,22 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -799,22 +799,22 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -831,32 +831,32 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -873,32 +873,32 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -925,22 +925,22 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -967,22 +967,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1009,12 +1009,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-05-28 16:51 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -715,12 +715,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -757,22 +757,22 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -799,22 +799,22 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -831,32 +831,32 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -873,32 +873,32 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -925,22 +925,22 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -967,22 +967,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1009,12 +1009,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-05-29 16:40 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -715,12 +715,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -757,22 +757,22 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -799,22 +799,22 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -831,32 +831,32 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -873,32 +873,32 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -925,22 +925,22 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -967,22 +967,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1009,12 +1009,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-05-30 14:26 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -715,12 +715,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -757,22 +757,22 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -799,22 +799,22 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -831,32 +831,32 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -873,32 +873,32 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -925,22 +925,22 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -967,22 +967,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1009,12 +1009,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-05-31 14:28 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Eventos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,106 +485,106 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-29T00:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-27T00:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>CAM 294 25 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-05-20T00:00:00</t>
+          <t>2026-05-26T00:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -594,17 +594,17 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Venda da Participação Societária na Stix</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -616,91 +616,91 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-05-18T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 1T26</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-05-15T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Alteração Estatuto Social</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-20T00:00:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -715,44 +715,44 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Venda da Participação Societária na Stix</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-18T00:00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -767,12 +767,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -784,37 +784,37 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -841,22 +841,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Convocação AGE</t>
-        </is>
-      </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -873,12 +873,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -893,12 +893,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -935,12 +935,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1036,17 +1036,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1061,12 +1061,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1078,101 +1078,101 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Alienação de Ativos HNT São Paulo</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Deferimento RJ</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1182,59 +1182,59 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Notícia veiculada na mídia</t>
+          <t>Alienação de Ativos HNT São Paulo</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+          <t>Apresentação de Resultado 1T26</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1246,42 +1246,168 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CVLB BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>16233389000155</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Deferimento RJ</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Notícia veiculada na mídia</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
           <t>2026-05-04T00:00:00</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>00776574000156</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Comunicado ao Mercado</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>CAM 268 24 - Desistência dos requerentes</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H20"/>
+  <autoFilter ref="A1:H23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza historico e state 2026-06-01 18:35 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -841,22 +841,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -888,17 +888,17 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -925,22 +925,22 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -957,32 +957,32 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1041,32 +1041,32 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1093,22 +1093,22 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1135,22 +1135,22 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-06-03 17:58 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -856,7 +856,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -883,22 +883,22 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -925,22 +925,22 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -957,32 +957,32 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -999,32 +999,32 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1051,22 +1051,22 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1098,17 +1098,17 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1135,22 +1135,22 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-06-06 14:26 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -831,32 +831,32 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -883,22 +883,22 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -930,17 +930,17 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -967,22 +967,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -999,32 +999,32 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1051,22 +1051,22 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1093,22 +1093,22 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-06-15 18:00 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Eventos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,64 +485,64 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-29T00:00:00</t>
+          <t>2026-06-13T00:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-27T00:00:00</t>
+          <t>2026-06-10T00:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -557,12 +557,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>CAM 294 25 Instauração da arbitragem</t>
+          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -574,17 +574,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-05-26T00:00:00</t>
+          <t>2026-05-29T00:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -604,91 +604,91 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-27T00:00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>CAM 294 25 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-26T00:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -700,37 +700,37 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-05-20T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Venda da Participação Societária na Stix</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -742,101 +742,101 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-05-18T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 1T26</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-05-15T00:00:00</t>
+          <t>2026-05-20T00:00:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Alteração Estatuto Social</t>
+          <t>Venda da Participação Societária na Stix</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-18T00:00:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -851,12 +851,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -868,17 +868,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -893,12 +893,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -925,22 +925,22 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -967,22 +967,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Convocação AGE</t>
-        </is>
-      </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1009,22 +1009,22 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1051,22 +1051,22 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1093,22 +1093,22 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1182,17 +1182,17 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Alienação de Ativos HNT São Paulo</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1204,101 +1204,101 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Deferimento RJ</t>
+          <t>Alienação de Ativos HNT São Paulo</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1308,17 +1308,17 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Notícia veiculada na mídia</t>
+          <t>Apresentação de Resultado 1T26</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1335,12 +1335,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1355,12 +1355,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+          <t>Deferimento RJ</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1372,42 +1372,126 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Notícia veiculada na mídia</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>2026-05-04T00:00:00</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>00776574000156</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>Comunicado ao Mercado</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>CAM 268 24 - Desistência dos requerentes</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H23"/>
+  <autoFilter ref="A1:H25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza historico e state 2026-06-16 17:59 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -925,22 +925,22 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -967,12 +967,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -982,7 +982,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -999,12 +999,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1019,12 +1019,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1051,22 +1051,22 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1098,17 +1098,17 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1135,22 +1135,22 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1167,32 +1167,32 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1229,12 +1229,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-06-17 16:35 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -930,17 +930,17 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -977,12 +977,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -999,32 +999,32 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1051,22 +1051,22 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1083,12 +1083,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1103,12 +1103,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1135,22 +1135,22 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1177,12 +1177,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1219,22 +1219,22 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-06-18 16:24 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -915,12 +915,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -935,12 +935,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -967,22 +967,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1009,12 +1009,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1024,7 +1024,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1051,22 +1051,22 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1083,32 +1083,32 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1135,22 +1135,22 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1187,12 +1187,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1224,17 +1224,17 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-06-20 15:01 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -915,32 +915,32 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -972,17 +972,17 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1051,22 +1051,22 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1093,12 +1093,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1135,22 +1135,22 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1177,22 +1177,22 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1209,12 +1209,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1229,12 +1229,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-06-21 15:09 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Eventos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,12 +485,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00</t>
+          <t>2026-06-17T00:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -505,34 +505,34 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00</t>
+          <t>2026-06-16T00:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -547,128 +547,128 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
+          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-05-29T00:00:00</t>
+          <t>2026-06-15T00:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>AGE 15/06 - Ata</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-05-27T00:00:00</t>
+          <t>2026-06-13T00:00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>CAM 294 25 Instauração da arbitragem</t>
+          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-05-26T00:00:00</t>
+          <t>2026-06-10T00:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -678,71 +678,71 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-29T00:00:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-27T00:00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -757,44 +757,44 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>CAM 294 25 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-05-20T00:00:00</t>
+          <t>2026-05-26T00:00:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -804,17 +804,17 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Venda da Participação Societária na Stix</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -826,91 +826,91 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-05-18T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 1T26</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-05-15T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Alteração Estatuto Social</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-20T00:00:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -925,44 +925,44 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Venda da Participação Societária na Stix</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-18T00:00:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -977,12 +977,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -994,17 +994,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1019,12 +1019,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1041,32 +1041,32 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1093,22 +1093,22 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1177,22 +1177,22 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1209,32 +1209,32 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1246,17 +1246,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1266,17 +1266,17 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Alienação de Ativos HNT São Paulo</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1288,59 +1288,59 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1355,34 +1355,34 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Deferimento RJ</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1392,59 +1392,59 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Notícia veiculada na mídia</t>
+          <t>Alienação de Ativos HNT São Paulo</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+          <t>Apresentação de Resultado 1T26</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1456,42 +1456,168 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>CVLB BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>16233389000155</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Deferimento RJ</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Notícia veiculada na mídia</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>2026-05-04T00:00:00</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>00776574000156</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>Comunicado ao Mercado</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>CAM 268 24 - Desistência dos requerentes</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H25"/>
+  <autoFilter ref="A1:H28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza historico e state 2026-06-22 17:27 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -831,32 +831,32 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -873,32 +873,32 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1041,32 +1041,32 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1093,22 +1093,22 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1135,22 +1135,22 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1177,22 +1177,22 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1209,32 +1209,32 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1261,22 +1261,22 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1303,22 +1303,22 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1345,22 +1345,22 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-06-23 15:44 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -831,32 +831,32 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -873,32 +873,32 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1041,32 +1041,32 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1093,22 +1093,22 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1135,22 +1135,22 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1177,22 +1177,22 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1209,32 +1209,32 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1261,22 +1261,22 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1303,22 +1303,22 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1345,22 +1345,22 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-06-24 15:31 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -831,32 +831,32 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -873,32 +873,32 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1041,32 +1041,32 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1093,22 +1093,22 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1135,22 +1135,22 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1177,22 +1177,22 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1209,32 +1209,32 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1261,22 +1261,22 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1303,22 +1303,22 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1345,22 +1345,22 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-06-25 15:37 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -831,32 +831,32 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -873,32 +873,32 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1041,32 +1041,32 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1093,22 +1093,22 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1135,22 +1135,22 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1177,22 +1177,22 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1209,32 +1209,32 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1261,22 +1261,22 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1303,22 +1303,22 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1345,22 +1345,22 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-06-28 14:45 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Eventos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,12 +485,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-17T00:00:00</t>
+          <t>2026-06-26T00:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -520,19 +520,19 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-16T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -547,34 +547,34 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-15T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -589,34 +589,34 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Ata</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00</t>
+          <t>2026-06-17T00:00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -631,34 +631,34 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00</t>
+          <t>2026-06-16T00:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -673,128 +673,128 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
+          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-05-29T00:00:00</t>
+          <t>2026-06-15T00:00:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>AGE 15/06 - Ata</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-05-27T00:00:00</t>
+          <t>2026-06-13T00:00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>CAM 294 25 Instauração da arbitragem</t>
+          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-05-26T00:00:00</t>
+          <t>2026-06-10T00:00:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -804,71 +804,71 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-29T00:00:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-27T00:00:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -883,44 +883,44 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>CAM 294 25 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-05-20T00:00:00</t>
+          <t>2026-05-26T00:00:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -930,17 +930,17 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Venda da Participação Societária na Stix</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -952,101 +952,101 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-05-18T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 1T26</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-05-15T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Alteração Estatuto Social</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-20T00:00:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1056,39 +1056,39 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Venda da Participação Societária na Stix</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-18T00:00:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1098,17 +1098,17 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1120,17 +1120,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1145,12 +1145,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1177,12 +1177,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1219,22 +1219,22 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1261,22 +1261,22 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1303,22 +1303,22 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1345,22 +1345,22 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Convocação AGE</t>
-        </is>
-      </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1372,17 +1372,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1397,12 +1397,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Alienação de Ativos HNT São Paulo</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1414,17 +1414,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1439,76 +1439,76 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Deferimento RJ</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1518,59 +1518,59 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Notícia veiculada na mídia</t>
+          <t>Alienação de Ativos HNT São Paulo</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+          <t>Apresentação de Resultado 1T26</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1582,42 +1582,168 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>CVLB BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>16233389000155</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Deferimento RJ</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Notícia veiculada na mídia</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>2026-05-04T00:00:00</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>00776574000156</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>Comunicado ao Mercado</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>CAM 268 24 - Desistência dos requerentes</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H28"/>
+  <autoFilter ref="A1:H31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza historico e state 2026-07-06 16:16 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Eventos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,54 +485,54 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-26T00:00:00</t>
+          <t>2026-07-03T00:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Conclusão da Venda da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-07-02T00:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -557,66 +557,66 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>Conclusão Operação Stix</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-06-30T00:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-17T00:00:00</t>
+          <t>2026-06-26T00:00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -646,19 +646,19 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-16T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -673,34 +673,34 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-06-15T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -715,34 +715,34 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Ata</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00</t>
+          <t>2026-06-17T00:00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -757,34 +757,34 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00</t>
+          <t>2026-06-16T00:00:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -799,128 +799,128 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
+          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-05-29T00:00:00</t>
+          <t>2026-06-15T00:00:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>AGE 15/06 - Ata</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-05-27T00:00:00</t>
+          <t>2026-06-13T00:00:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>CAM 294 25 Instauração da arbitragem</t>
+          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-05-26T00:00:00</t>
+          <t>2026-06-10T00:00:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -930,71 +930,71 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-29T00:00:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-27T00:00:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1009,44 +1009,44 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>CAM 294 25 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-05-20T00:00:00</t>
+          <t>2026-05-26T00:00:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1056,17 +1056,17 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Venda da Participação Societária na Stix</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1078,49 +1078,49 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-05-18T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 1T26</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-05-15T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1145,24 +1145,24 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Alteração Estatuto Social</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-20T00:00:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1177,64 +1177,64 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Venda da Participação Societária na Stix</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-18T00:00:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1246,17 +1246,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1271,12 +1271,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1293,12 +1293,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1313,12 +1313,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1355,12 +1355,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1387,22 +1387,22 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1419,12 +1419,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1434,17 +1434,17 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1481,12 +1481,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1498,17 +1498,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1518,17 +1518,17 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Alienação de Ativos HNT São Paulo</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1540,101 +1540,101 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 1T26</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Deferimento RJ</t>
-        </is>
-      </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1644,59 +1644,59 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Notícia veiculada na mídia</t>
+          <t>Alienação de Ativos HNT São Paulo</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+          <t>Apresentação de Resultado 1T26</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1708,42 +1708,168 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>CVLB BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>16233389000155</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Deferimento RJ</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Notícia veiculada na mídia</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
           <t>2026-05-04T00:00:00</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>00776574000156</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>Comunicado ao Mercado</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>CAM 268 24 - Desistência dos requerentes</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H31"/>
+  <autoFilter ref="A1:H34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza historico e state 2026-07-13 15:39 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Eventos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,12 +485,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-07-13T15:39:29</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-03T00:00:00</t>
+          <t>2026-07-09T00:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -505,22 +505,22 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Conclusão da Venda da UPI Uni.Co</t>
+          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -532,37 +532,37 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-02T00:00:00</t>
+          <t>2026-07-03T00:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Conclusão Operação Stix</t>
+          <t>Conclusão da Venda da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -574,17 +574,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-30T00:00:00</t>
+          <t>2026-07-02T00:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -594,39 +594,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Conclusão Operação Stix</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-26T00:00:00</t>
+          <t>2026-06-30T00:00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -636,17 +636,17 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-06-26T00:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -678,17 +678,17 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -715,34 +715,34 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-06-17T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -757,12 +757,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -772,7 +772,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -784,7 +784,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-06-16T00:00:00</t>
+          <t>2026-06-17T00:00:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -799,22 +799,22 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-15T00:00:00</t>
+          <t>2026-06-16T00:00:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -851,24 +851,24 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Ata</t>
+          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00</t>
+          <t>2026-06-15T00:00:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -893,12 +893,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
+          <t>AGE 15/06 - Ata</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -910,7 +910,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00</t>
+          <t>2026-06-13T00:00:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -925,44 +925,44 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
+          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-05-29T00:00:00</t>
+          <t>2026-06-10T00:00:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -972,17 +972,17 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -994,17 +994,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-05-27T00:00:00</t>
+          <t>2026-05-29T00:00:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1014,17 +1014,17 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>CAM 294 25 Instauração da arbitragem</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1036,17 +1036,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-05-26T00:00:00</t>
+          <t>2026-05-27T00:00:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1056,59 +1056,59 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>CAM 294 25 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-26T00:00:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1125,32 +1125,32 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1162,37 +1162,37 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-05-20T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Venda da Participação Societária na Stix</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1204,17 +1204,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-05-18T00:00:00</t>
+          <t>2026-05-20T00:00:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1224,59 +1224,59 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 1T26</t>
+          <t>Venda da Participação Societária na Stix</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-05-15T00:00:00</t>
+          <t>2026-05-18T00:00:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Alteração Estatuto Social</t>
+          <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1288,37 +1288,37 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1335,32 +1335,32 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1402,7 +1402,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1429,22 +1429,22 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1471,22 +1471,22 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1513,22 +1513,22 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1555,22 +1555,22 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1597,22 +1597,22 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1624,37 +1624,37 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Alienação de Ativos HNT São Paulo</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1671,12 +1671,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1686,59 +1686,59 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 1T26</t>
+          <t>Alienação de Ativos HNT São Paulo</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Deferimento RJ</t>
+          <t>Apresentação de Resultado 1T26</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1755,32 +1755,32 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Notícia veiculada na mídia</t>
+          <t>Deferimento RJ</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1807,22 +1807,22 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+          <t>Notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1834,42 +1834,84 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
           <t>2026-05-04T00:00:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>00776574000156</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>Comunicado ao Mercado</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>CAM 268 24 - Desistência dos requerentes</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H35" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H34"/>
+  <autoFilter ref="A1:H35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza historico e state 2026-07-20 15:06 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Eventos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,22 +485,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-13T15:39:29</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-09T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -510,81 +510,81 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-03T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Conclusão da Venda da UPI Uni.Co</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-07-13T15:39:29</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-02T00:00:00</t>
+          <t>2026-07-09T00:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -599,12 +599,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Conclusão Operação Stix</t>
+          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-30T00:00:00</t>
+          <t>2026-07-03T00:00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -631,34 +631,34 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Conclusão da Venda da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-26T00:00:00</t>
+          <t>2026-07-02T00:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -678,39 +678,39 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Conclusão Operação Stix</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-06-30T00:00:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -720,17 +720,17 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-06-26T00:00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -757,12 +757,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -772,19 +772,19 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-06-17T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -799,12 +799,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -814,19 +814,19 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-16T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -841,22 +841,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -868,7 +868,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-06-15T00:00:00</t>
+          <t>2026-06-17T00:00:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -883,34 +883,34 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Ata</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00</t>
+          <t>2026-06-16T00:00:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -935,24 +935,24 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
+          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00</t>
+          <t>2026-06-15T00:00:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -967,86 +967,86 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
+          <t>AGE 15/06 - Ata</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-05-29T00:00:00</t>
+          <t>2026-06-13T00:00:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-05-27T00:00:00</t>
+          <t>2026-06-10T00:00:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1061,12 +1061,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>CAM 294 25 Instauração da arbitragem</t>
+          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1078,17 +1078,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-05-26T00:00:00</t>
+          <t>2026-05-29T00:00:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1108,19 +1108,19 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-27T00:00:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1135,64 +1135,64 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>CAM 294 25 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-26T00:00:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1204,37 +1204,37 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-05-20T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Venda da Participação Societária na Stix</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1246,101 +1246,101 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-05-18T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 1T26</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-05-15T00:00:00</t>
+          <t>2026-05-20T00:00:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Alteração Estatuto Social</t>
+          <t>Venda da Participação Societária na Stix</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-18T00:00:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1355,12 +1355,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1372,17 +1372,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1397,12 +1397,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1444,7 +1444,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1471,22 +1471,22 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1513,22 +1513,22 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1555,22 +1555,22 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1597,22 +1597,22 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1639,22 +1639,22 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1666,37 +1666,37 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Alienação de Ativos HNT São Paulo</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1708,17 +1708,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1733,76 +1733,76 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Deferimento RJ</t>
+          <t>Alienação de Ativos HNT São Paulo</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1812,17 +1812,17 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Notícia veiculada na mídia</t>
+          <t>Apresentação de Resultado 1T26</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1839,12 +1839,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1859,12 +1859,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+          <t>Deferimento RJ</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1876,42 +1876,126 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Notícia veiculada na mídia</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t>2026-05-04T00:00:00</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>00776574000156</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>Comunicado ao Mercado</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>CAM 268 24 - Desistência dos requerentes</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H35"/>
+  <autoFilter ref="A1:H37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza historico e state 2026-07-21 15:00 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -799,22 +799,22 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -841,22 +841,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1209,32 +1209,32 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1251,32 +1251,32 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1429,22 +1429,22 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1461,32 +1461,32 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1513,22 +1513,22 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1555,22 +1555,22 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1597,22 +1597,22 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1639,22 +1639,22 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1681,22 +1681,22 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1713,32 +1713,32 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-07-22 15:00 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -799,22 +799,22 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -841,22 +841,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1209,32 +1209,32 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1251,32 +1251,32 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1429,22 +1429,22 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1461,32 +1461,32 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1513,22 +1513,22 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1555,22 +1555,22 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1597,22 +1597,22 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1639,22 +1639,22 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1671,32 +1671,32 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1723,22 +1723,22 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-07-24 14:49 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -799,22 +799,22 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -841,22 +841,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1209,32 +1209,32 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1251,32 +1251,32 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1429,22 +1429,22 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1471,22 +1471,22 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1503,32 +1503,32 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1555,22 +1555,22 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1597,22 +1597,22 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1639,22 +1639,22 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1671,32 +1671,32 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1723,22 +1723,22 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-07-25 14:27 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -799,22 +799,22 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -841,22 +841,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1209,32 +1209,32 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1251,32 +1251,32 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1429,22 +1429,22 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1471,22 +1471,22 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1503,32 +1503,32 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1555,22 +1555,22 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1597,22 +1597,22 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1629,32 +1629,32 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1681,22 +1681,22 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1723,22 +1723,22 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-07-26 14:26 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Eventos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,22 +485,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-07-26T14:26:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-07-20T00:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -510,17 +510,17 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Alteração na Administração da Companhia</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -569,22 +569,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-13T15:39:29</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-09T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -594,29 +594,29 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-07-13T15:39:29</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-03T00:00:00</t>
+          <t>2026-07-09T00:00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -631,22 +631,22 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Conclusão da Venda da UPI Uni.Co</t>
+          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -658,37 +658,37 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-02T00:00:00</t>
+          <t>2026-07-03T00:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Conclusão Operação Stix</t>
+          <t>Conclusão da Venda da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -700,17 +700,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-06-30T00:00:00</t>
+          <t>2026-07-02T00:00:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -720,39 +720,39 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Conclusão Operação Stix</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-06-26T00:00:00</t>
+          <t>2026-06-30T00:00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -762,17 +762,17 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -784,7 +784,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-06-26T00:00:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -799,12 +799,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -841,34 +841,34 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-06-17T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -888,17 +888,17 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -910,7 +910,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-06-16T00:00:00</t>
+          <t>2026-06-17T00:00:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -925,22 +925,22 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-06-15T00:00:00</t>
+          <t>2026-06-16T00:00:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -977,24 +977,24 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Ata</t>
+          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00</t>
+          <t>2026-06-15T00:00:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1019,12 +1019,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
+          <t>AGE 15/06 - Ata</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00</t>
+          <t>2026-06-13T00:00:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1051,44 +1051,44 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
+          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-05-29T00:00:00</t>
+          <t>2026-06-10T00:00:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1098,17 +1098,17 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1120,17 +1120,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-05-27T00:00:00</t>
+          <t>2026-05-29T00:00:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1140,17 +1140,17 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>CAM 294 25 Instauração da arbitragem</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1162,17 +1162,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-05-26T00:00:00</t>
+          <t>2026-05-27T00:00:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1182,59 +1182,59 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>CAM 294 25 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-26T00:00:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1288,37 +1288,37 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-05-20T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Venda da Participação Societária na Stix</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1330,17 +1330,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-05-18T00:00:00</t>
+          <t>2026-05-20T00:00:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1350,59 +1350,59 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 1T26</t>
+          <t>Venda da Participação Societária na Stix</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-05-15T00:00:00</t>
+          <t>2026-05-18T00:00:00</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Alteração Estatuto Social</t>
+          <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1414,37 +1414,37 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1471,22 +1471,22 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1523,12 +1523,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1570,7 +1570,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1597,22 +1597,22 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1629,32 +1629,32 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1671,12 +1671,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1691,12 +1691,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1750,17 +1750,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1770,17 +1770,17 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Alienação de Ativos HNT São Paulo</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1797,12 +1797,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1812,59 +1812,59 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 1T26</t>
+          <t>Alienação de Ativos HNT São Paulo</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Deferimento RJ</t>
+          <t>Apresentação de Resultado 1T26</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1881,32 +1881,32 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Notícia veiculada na mídia</t>
+          <t>Deferimento RJ</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1933,22 +1933,22 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+          <t>Notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1960,42 +1960,84 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
           <t>2026-05-04T00:00:00</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>00776574000156</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>Comunicado ao Mercado</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>CAM 268 24 - Desistência dos requerentes</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H37"/>
+  <autoFilter ref="A1:H38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza historico e state 2026-07-27 15:38 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -537,32 +537,32 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -579,32 +579,32 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1251,32 +1251,32 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1293,32 +1293,32 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1471,22 +1471,22 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1513,22 +1513,22 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1555,22 +1555,22 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1587,32 +1587,32 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1639,22 +1639,22 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1671,32 +1671,32 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1723,22 +1723,22 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Convocação AGE</t>
-        </is>
-      </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1770,17 +1770,17 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-07-28 15:15 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -537,32 +537,32 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -579,32 +579,32 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1251,32 +1251,32 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1293,32 +1293,32 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1471,22 +1471,22 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1518,17 +1518,17 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1555,22 +1555,22 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Convocação AGE</t>
-        </is>
-      </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1587,32 +1587,32 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1629,32 +1629,32 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1681,22 +1681,22 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1723,22 +1723,22 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1765,22 +1765,22 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-07-29 15:30 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -537,32 +537,32 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -579,32 +579,32 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1251,32 +1251,32 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1293,32 +1293,32 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1461,32 +1461,32 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1513,22 +1513,22 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1555,22 +1555,22 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1597,22 +1597,22 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1629,32 +1629,32 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1681,22 +1681,22 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Convocação AGE</t>
-        </is>
-      </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1728,17 +1728,17 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1765,22 +1765,22 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-02 14:25 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Eventos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$43</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,138 +485,138 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-26T14:26:00</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-20T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Alteração na Administração da Companhia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-13T15:39:29</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-09T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -631,34 +631,34 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-03T00:00:00</t>
+          <t>2026-07-27T00:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -673,44 +673,44 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Conclusão da Venda da UPI Uni.Co</t>
+          <t>CAM 236 23 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-07-26T14:26:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-02T00:00:00</t>
+          <t>2026-07-20T00:00:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -725,66 +725,66 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Conclusão Operação Stix</t>
+          <t>Alteração na Administração da Companhia</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-06-30T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-06-26T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -804,113 +804,113 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-13T15:39:29</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-07-09T00:00:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-07-03T00:00:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>Conclusão da Venda da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-06-17T00:00:00</t>
+          <t>2026-07-02T00:00:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -930,71 +930,71 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Conclusão Operação Stix</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-06-16T00:00:00</t>
+          <t>2026-06-30T00:00:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-15T00:00:00</t>
+          <t>2026-06-26T00:00:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1009,34 +1009,34 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Ata</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1051,34 +1051,34 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1093,44 +1093,44 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-05-29T00:00:00</t>
+          <t>2026-06-17T00:00:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1140,207 +1140,207 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-05-27T00:00:00</t>
+          <t>2026-06-16T00:00:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>CAM 294 25 Instauração da arbitragem</t>
+          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-05-26T00:00:00</t>
+          <t>2026-06-15T00:00:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>AGE 15/06 - Ata</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-06-13T00:00:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-06-10T00:00:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-05-20T00:00:00</t>
+          <t>2026-05-29T00:00:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1350,39 +1350,39 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Venda da Participação Societária na Stix</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-05-18T00:00:00</t>
+          <t>2026-05-27T00:00:00</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1392,71 +1392,71 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 1T26</t>
+          <t>CAM 294 25 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-05-15T00:00:00</t>
+          <t>2026-05-26T00:00:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Alteração Estatuto Social</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1471,76 +1471,76 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-20T00:00:00</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1560,59 +1560,59 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Venda da Participação Societária na Stix</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-18T00:00:00</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1624,17 +1624,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1649,12 +1649,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1691,12 +1691,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1723,22 +1723,22 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1765,22 +1765,22 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1792,37 +1792,37 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Alienação de Ativos HNT São Paulo</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1834,101 +1834,101 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 1T26</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Deferimento RJ</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1938,29 +1938,29 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Notícia veiculada na mídia</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1975,69 +1975,279 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
-        </is>
-      </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-05-13T00:00:00</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>00776574000156</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Alienação de Ativos HNT São Paulo</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-05-13T00:00:00</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>GRUPO CASAS BAHIA S.A.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>33041260065290</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Apresentações a analistas/agentes do mercado</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Apresentação de Resultado 1T26</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>2026-05-13T19:28:37</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>CVLB BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>16233389000155</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Deferimento RJ</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Notícia veiculada na mídia</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
         <is>
           <t>2026-05-04T00:00:00</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>00776574000156</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>Comunicado ao Mercado</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="G43" t="inlineStr">
         <is>
           <t>CAM 268 24 - Desistência dos requerentes</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H38"/>
+  <autoFilter ref="A1:H43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-03 15:39 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -1681,22 +1681,22 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1713,32 +1713,32 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1770,17 +1770,17 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1807,22 +1807,22 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1849,22 +1849,22 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1896,17 +1896,17 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1923,32 +1923,32 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1975,22 +1975,22 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-04 15:21 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -1681,22 +1681,22 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1713,32 +1713,32 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1770,17 +1770,17 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1807,22 +1807,22 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1849,22 +1849,22 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1896,17 +1896,17 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1923,32 +1923,32 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1975,22 +1975,22 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-05 15:10 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -1681,22 +1681,22 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1713,32 +1713,32 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1770,17 +1770,17 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1807,22 +1807,22 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1849,22 +1849,22 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1896,17 +1896,17 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1923,32 +1923,32 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1975,22 +1975,22 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-06 15:09 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -1681,22 +1681,22 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1713,32 +1713,32 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1770,17 +1770,17 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1807,22 +1807,22 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1849,22 +1849,22 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1896,17 +1896,17 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1923,32 +1923,32 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1975,22 +1975,22 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-07 14:08 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -1681,22 +1681,22 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1713,32 +1713,32 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1770,17 +1770,17 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1807,22 +1807,22 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1849,22 +1849,22 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1896,17 +1896,17 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1923,32 +1923,32 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1975,22 +1975,22 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-09 13:44 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Eventos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,12 +485,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-07T00:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -505,64 +505,64 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Conclusão do procedimento de ajuste de preço da alienação da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1554573&amp;numSequencia=1079279&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-04T00:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>Apresentação de Resultado - 2T26</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1552160&amp;numSequencia=1076866&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -599,12 +599,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -641,12 +641,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-27T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -673,128 +673,128 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>CAM 236 23 Instauração da arbitragem</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-26T14:26:00</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-20T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Alteração na Administração da Companhia</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-07-27T00:00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>CAM 236 23 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-07-26T14:26:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-07-20T00:00:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -804,39 +804,39 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Alteração na Administração da Companhia</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-07-13T15:39:29</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-09T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -846,81 +846,81 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-03T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Conclusão da Venda da UPI Uni.Co</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-07-13T15:39:29</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-02T00:00:00</t>
+          <t>2026-07-09T00:00:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -935,12 +935,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Conclusão Operação Stix</t>
+          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-06-30T00:00:00</t>
+          <t>2026-07-03T00:00:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -967,34 +967,34 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Conclusão da Venda da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-26T00:00:00</t>
+          <t>2026-07-02T00:00:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1014,39 +1014,39 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Conclusão Operação Stix</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-06-30T00:00:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1056,17 +1056,17 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-06-26T00:00:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1093,12 +1093,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1108,19 +1108,19 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-06-17T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1135,12 +1135,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1150,19 +1150,19 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-06-16T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1177,22 +1177,22 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-06-15T00:00:00</t>
+          <t>2026-06-17T00:00:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1219,34 +1219,34 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Ata</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00</t>
+          <t>2026-06-16T00:00:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1271,24 +1271,24 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
+          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00</t>
+          <t>2026-06-15T00:00:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1303,86 +1303,86 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
+          <t>AGE 15/06 - Ata</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-05-29T00:00:00</t>
+          <t>2026-06-13T00:00:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-05-27T00:00:00</t>
+          <t>2026-06-10T00:00:00</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1397,12 +1397,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>CAM 294 25 Instauração da arbitragem</t>
+          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1414,17 +1414,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-05-26T00:00:00</t>
+          <t>2026-05-29T00:00:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1444,19 +1444,19 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-27T00:00:00</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1471,64 +1471,64 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>CAM 294 25 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-26T00:00:00</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1540,37 +1540,37 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-05-20T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Venda da Participação Societária na Stix</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1582,121 +1582,121 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-05-18T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 1T26</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-05-15T00:00:00</t>
+          <t>2026-05-20T00:00:00</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Alteração Estatuto Social</t>
+          <t>Venda da Participação Societária na Stix</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-18T00:00:00</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1708,37 +1708,37 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1765,22 +1765,22 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1797,32 +1797,32 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1849,22 +1849,22 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1891,22 +1891,22 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1943,12 +1943,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1975,22 +1975,22 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2002,37 +2002,37 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Alienação de Ativos HNT São Paulo</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2044,101 +2044,101 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Deferimento RJ</t>
+          <t>Alienação de Ativos HNT São Paulo</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2148,17 +2148,17 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Notícia veiculada na mídia</t>
+          <t>Apresentação de Resultado 1T26</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2175,12 +2175,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2195,12 +2195,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+          <t>Deferimento RJ</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2212,42 +2212,126 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Notícia veiculada na mídia</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
           <t>2026-05-04T00:00:00</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>00776574000156</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>Comunicado ao Mercado</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="G45" t="inlineStr">
         <is>
           <t>CAM 268 24 - Desistência dos requerentes</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="H45" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H43"/>
+  <autoFilter ref="A1:H45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-11 14:16 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -1765,22 +1765,22 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1797,32 +1797,32 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1849,22 +1849,22 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1891,22 +1891,22 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1933,22 +1933,22 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1980,17 +1980,17 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2007,32 +2007,32 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2059,12 +2059,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-12 14:17 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -1765,22 +1765,22 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1807,12 +1807,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1839,32 +1839,32 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1896,17 +1896,17 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1933,22 +1933,22 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1975,22 +1975,22 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2007,32 +2007,32 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2059,22 +2059,22 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-14 14:12 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -1765,22 +1765,22 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1807,22 +1807,22 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -1839,32 +1839,32 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1891,22 +1891,22 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1938,17 +1938,17 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1965,32 +1965,32 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2017,12 +2017,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2059,22 +2059,22 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-15 13:25 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -1770,17 +1770,17 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1807,22 +1807,22 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1849,12 +1849,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1881,32 +1881,32 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1933,22 +1933,22 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1965,32 +1965,32 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2017,22 +2017,22 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2059,22 +2059,22 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-16 13:26 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Eventos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$53</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,22 +485,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-09T13:44:03</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-07T00:00:00</t>
+          <t>2026-08-16T00:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -510,29 +510,29 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Conclusão do procedimento de ajuste de preço da alienação da UPI Uni.Co</t>
+          <t>Apresentação de Resultado 2T26</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1554573&amp;numSequencia=1079279&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558370&amp;numSequencia=1083076&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-09T13:44:03</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-04T00:00:00</t>
+          <t>2026-08-14T00:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -552,29 +552,29 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 2T26</t>
+          <t>Disponibilização Term Sheet na CVM</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1552160&amp;numSequencia=1076866&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558099&amp;numSequencia=1082805&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-13T00:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -589,34 +589,34 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-13T00:00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -631,212 +631,212 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultados 2T26</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-12T00:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Term Sheet das debêntures do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556765&amp;numSequencia=1081471&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-11T00:00:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-27T00:00:00</t>
+          <t>2026-08-11T00:00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>CAM 236 23 Instauração da arbitragem</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-26T14:26:00</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-07-20T00:00:00</t>
+          <t>2026-08-10T00:00:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Alteração na Administração da Companhia</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1555456&amp;numSequencia=1080162&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-08-07T00:00:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -846,71 +846,71 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Conclusão do procedimento de ajuste de preço da alienação da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1554573&amp;numSequencia=1079279&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-08-04T00:00:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>Apresentação de Resultado - 2T26</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1552160&amp;numSequencia=1076866&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-07-13T15:39:29</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-09T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -925,34 +925,34 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-03T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -967,76 +967,76 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Conclusão da Venda da UPI Uni.Co</t>
-        </is>
-      </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-02T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Conclusão Operação Stix</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-06-30T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1051,44 +1051,44 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-06-26T00:00:00</t>
+          <t>2026-07-27T00:00:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1098,71 +1098,71 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>CAM 236 23 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-26T14:26:00</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-07-20T00:00:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alteração na Administração da Companhia</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1182,155 +1182,155 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-06-17T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-07-13T15:39:29</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-06-16T00:00:00</t>
+          <t>2026-07-09T00:00:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
+          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-06-15T00:00:00</t>
+          <t>2026-07-03T00:00:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Ata</t>
+          <t>Conclusão da Venda da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00</t>
+          <t>2026-07-02T00:00:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1345,44 +1345,44 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
+          <t>Conclusão Operação Stix</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00</t>
+          <t>2026-06-30T00:00:00</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1392,39 +1392,39 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-05-29T00:00:00</t>
+          <t>2026-06-26T00:00:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1434,39 +1434,39 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-05-27T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1481,150 +1481,150 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>CAM 294 25 Instauração da arbitragem</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-05-26T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-06-17T00:00:00</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-06-16T00:00:00</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-05-20T00:00:00</t>
+          <t>2026-06-15T00:00:00</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1639,128 +1639,128 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Venda da Participação Societária na Stix</t>
+          <t>AGE 15/06 - Ata</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-05-18T00:00:00</t>
+          <t>2026-06-13T00:00:00</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 1T26</t>
+          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-05-15T00:00:00</t>
+          <t>2026-06-10T00:00:00</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Alteração Estatuto Social</t>
+          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-29T00:00:00</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1770,113 +1770,113 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-27T00:00:00</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>CAM 294 25 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-26T00:00:00</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1891,44 +1891,44 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1943,24 +1943,24 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-20T00:00:00</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1975,64 +1975,64 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Venda da Participação Societária na Stix</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-18T00:00:00</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2044,37 +2044,37 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2086,37 +2086,37 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Alienação de Ativos HNT São Paulo</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2128,59 +2128,59 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2195,24 +2195,24 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Deferimento RJ</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2227,111 +2227,447 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Notícia veiculada na mídia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Apresentações a analistas/agentes do mercado</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Apresentação de Resultado - 1T26</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Assembleia</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-05-13T00:00:00</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>GRUPO CASAS BAHIA S.A.</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>33041260065290</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Apresentações a analistas/agentes do mercado</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Apresentação de Resultado 1T26</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-05-13T00:00:00</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>00776574000156</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Alienação de Ativos HNT São Paulo</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>2026-05-13T19:28:37</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Notícia veiculada na mídia</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>CVLB BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>16233389000155</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Deferimento RJ</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
         <is>
           <t>2026-05-04T00:00:00</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>00776574000156</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Comunicado ao Mercado</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G53" t="inlineStr">
         <is>
           <t>CAM 268 24 - Desistência dos requerentes</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="H53" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H45"/>
+  <autoFilter ref="A1:H53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-17 13:34 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -935,12 +935,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -977,12 +977,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2091,32 +2091,32 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2153,12 +2153,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2227,22 +2227,22 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2259,32 +2259,32 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2311,22 +2311,22 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2353,22 +2353,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2410,7 +2410,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-18 13:37 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -940,7 +940,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -982,7 +982,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1061,12 +1061,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2091,32 +2091,32 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2158,7 +2158,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2227,22 +2227,22 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2279,12 +2279,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2311,22 +2311,22 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2353,22 +2353,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2385,32 +2385,32 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-19 13:39 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -935,12 +935,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -977,12 +977,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2111,12 +2111,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2133,32 +2133,32 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2227,22 +2227,22 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2284,7 +2284,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2311,22 +2311,22 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2353,22 +2353,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2385,32 +2385,32 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-20 13:41 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -940,7 +940,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -982,7 +982,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1061,12 +1061,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2116,7 +2116,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2133,32 +2133,32 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2227,22 +2227,22 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2259,32 +2259,32 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2311,22 +2311,22 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2353,22 +2353,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2405,12 +2405,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-21 13:39 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -935,12 +935,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -977,12 +977,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2091,32 +2091,32 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2153,12 +2153,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2227,22 +2227,22 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2259,32 +2259,32 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2311,22 +2311,22 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2353,22 +2353,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2410,7 +2410,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-22 13:26 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -940,7 +940,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -982,7 +982,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1061,12 +1061,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2091,32 +2091,32 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2158,7 +2158,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2185,22 +2185,22 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2227,22 +2227,22 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2279,12 +2279,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2311,22 +2311,22 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2353,22 +2353,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2385,32 +2385,32 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-26 13:50 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Eventos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,22 +485,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-16T00:00:00</t>
+          <t>2026-08-24T00:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>CVLB BRASIL S.A EM RECUPERAÇÃO JUDICAL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -510,39 +510,39 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26</t>
+          <t>Resposta Ofício nº 241/2026-SLE, de 11/08/2026, sobre o andamento do proc. de recuperação judicial e, em especial, da apresentação de objeções ao Plano de Recuperação Judicial.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558370&amp;numSequencia=1083076&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560634&amp;numSequencia=1085340&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-14T00:00:00</t>
+          <t>2026-08-21T00:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -557,24 +557,24 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Disponibilização Term Sheet na CVM</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558099&amp;numSequencia=1082805&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-13T00:00:00</t>
+          <t>2026-08-21T00:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -589,44 +589,44 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-13T00:00:00</t>
+          <t>2026-08-18T00:00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -636,71 +636,71 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 2T26</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1559232&amp;numSequencia=1083938&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-08-12T00:00:00</t>
+          <t>2026-08-17T00:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Term Sheet das debêntures do Plano de Recuperação Extrajudicial</t>
+          <t>Apresentação de resultados 2T26</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556765&amp;numSequencia=1081471&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-11T00:00:00</t>
+          <t>2026-08-17T00:00:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -720,17 +720,17 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Alteração do Calendário de Eventos Corporativos</t>
+          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-08-11T00:00:00</t>
+          <t>2026-08-16T00:00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -757,22 +757,22 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado 2T26</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558370&amp;numSequencia=1083076&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -784,49 +784,49 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-08-10T00:00:00</t>
+          <t>2026-08-14T00:00:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Disponibilização Term Sheet na CVM</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1555456&amp;numSequencia=1080162&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558099&amp;numSequencia=1082805&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-09T13:44:03</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-08-07T00:00:00</t>
+          <t>2026-08-13T00:00:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -846,39 +846,39 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Conclusão do procedimento de ajuste de preço da alienação da UPI Uni.Co</t>
+          <t>Apresentação de Resultados 2T26</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1554573&amp;numSequencia=1079279&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-09T13:44:03</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-08-04T00:00:00</t>
+          <t>2026-08-13T00:00:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -888,155 +888,155 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 2T26</t>
+          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1552160&amp;numSequencia=1076866&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-12T00:00:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Term Sheet das debêntures do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556765&amp;numSequencia=1081471&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-11T00:00:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-11T00:00:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-10T00:00:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1051,34 +1051,34 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1555456&amp;numSequencia=1080162&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-27T00:00:00</t>
+          <t>2026-08-07T00:00:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1103,34 +1103,34 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>CAM 236 23 Instauração da arbitragem</t>
+          <t>Conclusão do procedimento de ajuste de preço da alienação da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1554573&amp;numSequencia=1079279&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-07-26T14:26:00</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-07-20T00:00:00</t>
+          <t>2026-08-04T00:00:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1140,113 +1140,113 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Alteração na Administração da Companhia</t>
+          <t>Apresentação de Resultado - 2T26</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1552160&amp;numSequencia=1076866&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-07-13T15:39:29</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-09T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1261,34 +1261,34 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-03T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1303,44 +1303,44 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Conclusão da Venda da UPI Uni.Co</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-02T00:00:00</t>
+          <t>2026-07-27T00:00:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1355,34 +1355,34 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Conclusão Operação Stix</t>
+          <t>CAM 236 23 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-07-26T14:26:00</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-06-30T00:00:00</t>
+          <t>2026-07-20T00:00:00</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1392,29 +1392,29 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Alteração na Administração da Companhia</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-06-26T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1434,155 +1434,155 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-13T15:39:29</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-07-09T00:00:00</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-06-17T00:00:00</t>
+          <t>2026-07-03T00:00:00</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Conclusão da Venda da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-06-16T00:00:00</t>
+          <t>2026-07-02T00:00:00</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1597,76 +1597,76 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
+          <t>Conclusão Operação Stix</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-06-15T00:00:00</t>
+          <t>2026-06-30T00:00:00</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Ata</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00</t>
+          <t>2026-06-26T00:00:00</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1681,34 +1681,34 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1733,76 +1733,76 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-05-29T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-05-27T00:00:00</t>
+          <t>2026-06-17T00:00:00</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1812,123 +1812,123 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>CAM 294 25 Instauração da arbitragem</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-05-26T00:00:00</t>
+          <t>2026-06-16T00:00:00</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-06-15T00:00:00</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>AGE 15/06 - Ata</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-06-13T00:00:00</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1943,24 +1943,24 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-05-20T00:00:00</t>
+          <t>2026-06-10T00:00:00</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1985,34 +1985,34 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Venda da Participação Societária na Stix</t>
+          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-05-18T00:00:00</t>
+          <t>2026-05-29T00:00:00</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2022,197 +2022,197 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 1T26</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-05-15T00:00:00</t>
+          <t>2026-05-27T00:00:00</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Alteração Estatuto Social</t>
+          <t>CAM 294 25 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-26T00:00:00</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-20T00:00:00</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2227,64 +2227,64 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Venda da Participação Societária na Stix</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-18T00:00:00</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2296,37 +2296,37 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2358,17 +2358,17 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2385,12 +2385,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2400,17 +2400,17 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2422,17 +2422,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2447,12 +2447,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2464,49 +2464,49 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Alienação de Ativos HNT São Paulo</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2521,34 +2521,34 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
-        </is>
-      </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2563,111 +2563,363 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Notícia veiculada na mídia</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Deferimento RJ</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Assembleia</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-05-13T00:00:00</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>GRUPO CASAS BAHIA S.A.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>33041260065290</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Apresentações a analistas/agentes do mercado</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Apresentação de Resultado 1T26</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-05-13T00:00:00</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>00776574000156</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Alienação de Ativos HNT São Paulo</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>2026-05-13T19:28:37</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Notícia veiculada na mídia</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>CVLB BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>16233389000155</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Deferimento RJ</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
         <is>
           <t>2026-05-04T00:00:00</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D59" t="inlineStr">
         <is>
           <t>00776574000156</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Comunicado ao Mercado</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="G59" t="inlineStr">
         <is>
           <t>CAM 268 24 - Desistência dos requerentes</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
+      <c r="H59" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H53"/>
+  <autoFilter ref="A1:H59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-27 22:43 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -537,32 +537,32 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -579,32 +579,32 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1187,12 +1187,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1234,7 +1234,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1271,12 +1271,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1723,22 +1723,22 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1765,22 +1765,22 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2133,32 +2133,32 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2175,32 +2175,32 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2353,22 +2353,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2395,22 +2395,22 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2427,32 +2427,32 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2479,22 +2479,22 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2521,22 +2521,22 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2563,22 +2563,22 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2595,32 +2595,32 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2647,22 +2647,22 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-28 22:50 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -537,32 +537,32 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -579,32 +579,32 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1229,12 +1229,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1313,12 +1313,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1723,22 +1723,22 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1765,22 +1765,22 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2133,32 +2133,32 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2175,32 +2175,32 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2353,22 +2353,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2395,22 +2395,22 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2427,32 +2427,32 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2479,22 +2479,22 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2521,22 +2521,22 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2563,22 +2563,22 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2595,32 +2595,32 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2647,22 +2647,22 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-29 16:56 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -537,32 +537,32 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -579,32 +579,32 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1187,12 +1187,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1234,7 +1234,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1271,12 +1271,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1723,22 +1723,22 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1765,22 +1765,22 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2133,32 +2133,32 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2175,32 +2175,32 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2353,22 +2353,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2395,22 +2395,22 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2427,32 +2427,32 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2479,22 +2479,22 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2521,22 +2521,22 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2563,22 +2563,22 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2595,32 +2595,32 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2647,22 +2647,22 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-08-30 17:07 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -537,32 +537,32 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -579,32 +579,32 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1229,12 +1229,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1313,12 +1313,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1723,22 +1723,22 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1765,22 +1765,22 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2133,32 +2133,32 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2175,32 +2175,32 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2353,22 +2353,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2395,22 +2395,22 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2427,32 +2427,32 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2479,22 +2479,22 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2521,22 +2521,22 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2563,22 +2563,22 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2595,32 +2595,32 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2647,22 +2647,22 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-01 17:06 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -537,32 +537,32 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -579,32 +579,32 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1187,12 +1187,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1234,7 +1234,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1271,12 +1271,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1723,22 +1723,22 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1765,22 +1765,22 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2133,32 +2133,32 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2175,32 +2175,32 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2353,22 +2353,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2395,22 +2395,22 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2427,32 +2427,32 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2479,22 +2479,22 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2521,22 +2521,22 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2563,22 +2563,22 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2595,32 +2595,32 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2647,22 +2647,22 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-02 16:57 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -537,32 +537,32 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -579,32 +579,32 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1229,12 +1229,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1313,12 +1313,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1723,22 +1723,22 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1765,22 +1765,22 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2133,32 +2133,32 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2175,32 +2175,32 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2353,22 +2353,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2395,22 +2395,22 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2427,32 +2427,32 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2479,22 +2479,22 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2521,22 +2521,22 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2563,22 +2563,22 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2595,32 +2595,32 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2647,22 +2647,22 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-06 15:56 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Eventos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$66</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,96 +485,96 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-24T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A EM RECUPERAÇÃO JUDICAL</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Resposta Ofício nº 241/2026-SLE, de 11/08/2026, sobre o andamento do proc. de recuperação judicial e, em especial, da apresentação de objeções ao Plano de Recuperação Judicial.</t>
+          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560634&amp;numSequencia=1085340&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-21T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564397&amp;numSequencia=1089103&amp;numVersao=5</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-21T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -589,128 +589,128 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-18T00:00:00</t>
+          <t>2026-09-01T00:00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1559232&amp;numSequencia=1083938&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-08-17T00:00:00</t>
+          <t>2026-09-01T00:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 2T26</t>
+          <t>Mapa de Votação Sintético Consolidado AGE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-17T00:00:00</t>
+          <t>2026-08-31T00:00:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -720,29 +720,29 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562894&amp;numSequencia=1087600&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-08-16T00:00:00</t>
+          <t>2026-08-31T00:00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -757,44 +757,44 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26</t>
+          <t>Deferimento de Tutela de Urgência na Recuperação Judicial</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558370&amp;numSequencia=1083076&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562849&amp;numSequencia=1087555&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-08-14T00:00:00</t>
+          <t>2026-08-24T00:00:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A EM RECUPERAÇÃO JUDICAL</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -804,29 +804,29 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Disponibilização Term Sheet na CVM</t>
+          <t>Resposta Ofício nº 241/2026-SLE, de 11/08/2026, sobre o andamento do proc. de recuperação judicial e, em especial, da apresentação de objeções ao Plano de Recuperação Judicial.</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558099&amp;numSequencia=1082805&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560634&amp;numSequencia=1085340&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-08-13T00:00:00</t>
+          <t>2026-08-21T00:00:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -841,44 +841,44 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 2T26</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-08-13T00:00:00</t>
+          <t>2026-08-21T00:00:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -893,66 +893,66 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-08-12T00:00:00</t>
+          <t>2026-08-18T00:00:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Term Sheet das debêntures do Plano de Recuperação Extrajudicial</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556765&amp;numSequencia=1081471&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1559232&amp;numSequencia=1083938&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-08-11T00:00:00</t>
+          <t>2026-08-17T00:00:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -972,59 +972,59 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Alteração do Calendário de Eventos Corporativos</t>
+          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-08-11T00:00:00</t>
+          <t>2026-08-17T00:00:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de resultados 2T26</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1036,59 +1036,59 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-08-10T00:00:00</t>
+          <t>2026-08-16T00:00:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Apresentação de Resultado 2T26</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1555456&amp;numSequencia=1080162&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558370&amp;numSequencia=1083076&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-09T13:44:03</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-08-07T00:00:00</t>
+          <t>2026-08-14T00:00:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1103,34 +1103,34 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Conclusão do procedimento de ajuste de preço da alienação da UPI Uni.Co</t>
+          <t>Disponibilização Term Sheet na CVM</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1554573&amp;numSequencia=1079279&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558099&amp;numSequencia=1082805&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-09T13:44:03</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-08-04T00:00:00</t>
+          <t>2026-08-13T00:00:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1140,29 +1140,29 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 2T26</t>
+          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1552160&amp;numSequencia=1076866&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-13T00:00:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1177,138 +1177,138 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultados 2T26</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-12T00:00:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>Term Sheet das debêntures do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556765&amp;numSequencia=1081471&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-11T00:00:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-11T00:00:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1318,19 +1318,19 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-27T00:00:00</t>
+          <t>2026-08-10T00:00:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1345,44 +1345,44 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>CAM 236 23 Instauração da arbitragem</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1555456&amp;numSequencia=1080162&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-26T14:26:00</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-07-20T00:00:00</t>
+          <t>2026-08-07T00:00:00</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1397,24 +1397,24 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Alteração na Administração da Companhia</t>
+          <t>Conclusão do procedimento de ajuste de preço da alienação da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1554573&amp;numSequencia=1079279&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-08-04T00:00:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1434,71 +1434,71 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Apresentação de Resultado - 2T26</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1552160&amp;numSequencia=1076866&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-07-13T15:39:29</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-09T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1513,34 +1513,34 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-03T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1555,76 +1555,76 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Conclusão da Venda da UPI Uni.Co</t>
-        </is>
-      </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-02T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Conclusão Operação Stix</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-06-30T00:00:00</t>
+          <t>2026-07-27T00:00:00</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1644,39 +1644,39 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>CAM 236 23 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-26T14:26:00</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-06-26T00:00:00</t>
+          <t>2026-07-20T00:00:00</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1686,71 +1686,71 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alteração na Administração da Companhia</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1765,44 +1765,44 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-07-13T15:39:29</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-06-17T00:00:00</t>
+          <t>2026-07-09T00:00:00</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1812,71 +1812,71 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-06-16T00:00:00</t>
+          <t>2026-07-03T00:00:00</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
+          <t>Conclusão da Venda da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-06-15T00:00:00</t>
+          <t>2026-07-02T00:00:00</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1891,76 +1891,76 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Ata</t>
+          <t>Conclusão Operação Stix</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00</t>
+          <t>2026-06-30T00:00:00</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00</t>
+          <t>2026-06-26T00:00:00</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1980,81 +1980,81 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-05-29T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-05-27T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2069,34 +2069,34 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>CAM 294 25 Instauração da arbitragem</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-05-26T00:00:00</t>
+          <t>2026-06-17T00:00:00</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2106,81 +2106,81 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-06-16T00:00:00</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-06-15T00:00:00</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2195,24 +2195,24 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>AGE 15/06 - Ata</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-05-20T00:00:00</t>
+          <t>2026-06-13T00:00:00</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2227,44 +2227,44 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Venda da Participação Societária na Stix</t>
+          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-05-18T00:00:00</t>
+          <t>2026-06-10T00:00:00</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2274,81 +2274,81 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 1T26</t>
+          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-05-15T00:00:00</t>
+          <t>2026-05-29T00:00:00</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Alteração Estatuto Social</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-27T00:00:00</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2358,39 +2358,39 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>CAM 294 25 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-26T00:00:00</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2400,29 +2400,29 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2437,44 +2437,44 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2489,24 +2489,24 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-20T00:00:00</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2521,64 +2521,64 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Venda da Participação Societária na Stix</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-18T00:00:00</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2590,17 +2590,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2615,12 +2615,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2647,12 +2647,12 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2662,7 +2662,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2674,17 +2674,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2699,12 +2699,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2716,49 +2716,49 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Alienação de Ativos HNT São Paulo</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2773,34 +2773,34 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
-        </is>
-      </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2820,39 +2820,39 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Notícia veiculada na mídia</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2867,59 +2867,353 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Deferimento RJ</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Assembleia</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-05-13T00:00:00</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>GRUPO CASAS BAHIA S.A.</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>33041260065290</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Apresentações a analistas/agentes do mercado</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Apresentação de Resultado 1T26</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-05-13T00:00:00</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>00776574000156</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Alienação de Ativos HNT São Paulo</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
           <t>2026-05-13T19:28:37</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Notícia veiculada na mídia</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>CVLB BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>16233389000155</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Deferimento RJ</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
         <is>
           <t>2026-05-04T00:00:00</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C66" t="inlineStr">
         <is>
           <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="D66" t="inlineStr">
         <is>
           <t>00776574000156</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Comunicado ao Mercado</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr">
+      <c r="G66" t="inlineStr">
         <is>
           <t>CAM 268 24 - Desistência dos requerentes</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr">
+      <c r="H66" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H59"/>
+  <autoFilter ref="A1:H66"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-07 18:02 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -1140,17 +1140,17 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
+          <t>Apresentação de Resultados 2T26</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1182,17 +1182,17 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 2T26</t>
+          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-08 17:00 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -1140,17 +1140,17 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 2T26</t>
+          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1182,17 +1182,17 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
+          <t>Apresentação de Resultados 2T26</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-09 16:58 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -1140,17 +1140,17 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
+          <t>Apresentação de Resultados 2T26</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1182,17 +1182,17 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 2T26</t>
+          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-10 16:51 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -1140,17 +1140,17 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 2T26</t>
+          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1182,17 +1182,17 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
+          <t>Apresentação de Resultados 2T26</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-11 16:50 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -1140,17 +1140,17 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
+          <t>Apresentação de Resultados 2T26</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1182,17 +1182,17 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 2T26</t>
+          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-12 15:57 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -1140,17 +1140,17 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 2T26</t>
+          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1182,17 +1182,17 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
+          <t>Apresentação de Resultados 2T26</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>